<commit_message>
Added template & sample finance tracker.
Expanded notes in README.
</commit_message>
<xml_diff>
--- a/SpendingTracker/FinanceTracker.xlsx
+++ b/SpendingTracker/FinanceTracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tyler\Desktop\Taxes\Fin\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tyler\GitLocal\miniportfolio\SpendingTracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0601748D-7F03-45E0-A3CA-59C6E28E0571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D4CB7F-6CF0-4087-A215-F26046282E79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>

</xml_diff>